<commit_message>
final stoch example added
</commit_message>
<xml_diff>
--- a/examples/genomics_results.xlsx
+++ b/examples/genomics_results.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="WS" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="RP" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="EEV" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="EV" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="metrics" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
@@ -1421,7 +1421,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EVPI</t>
+          <t>VPI</t>
         </is>
       </c>
       <c r="B5" t="n">

</xml_diff>